<commit_message>
Document callback advancement policy
</commit_message>
<xml_diff>
--- a/tests/fixtures/sample_event.xlsx
+++ b/tests/fixtures/sample_event.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -482,6 +482,7 @@
     <col width="19" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -510,6 +511,11 @@
           <t>notes</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>callback_advance_count</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -559,6 +565,9 @@
         <is>
           <t>Preliminary</t>
         </is>
+      </c>
+      <c r="F3" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>